<commit_message>
python main.py \   --image khb_dataset/train/images/02.jpg \   --labels khb_dataset/train/labels/02.txt \
</commit_message>
<xml_diff>
--- a/invoice_data.xlsx
+++ b/invoice_data.xlsx
@@ -422,8 +422,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,42 +471,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>70265202</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>91.03.2026</t>
+          <t>18.05.2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>6RA6</t>
+          <t>STT4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0009837418</t>
+          <t>0030077307</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>190369</t>
+          <t>100569</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>-8271</t>
+          <t>3A-5089</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KHB-Brewery-&gt;R4-Bavel</t>
+          <t>KHB-Brewery-&gt;R6-Chamka Leu</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>WF11-F'G Warehouse</t>
+          <t>WF11-FG Warehouse</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
multi image detect support python main.py \   --image_path "images" \   --conf 0.25
</commit_message>
<xml_diff>
--- a/invoice_data.xlsx
+++ b/invoice_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -421,9 +421,6 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,61 +449,15 @@
           <t>Vender Code</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Vehicle Code</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Route</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Warehouse</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>70265202</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>18.05.2026</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>STT4</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0030077307</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>100569</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>3A-5089</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>KHB-Brewery-&gt;R6-Chamka Leu</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>WF11-FG Warehouse</t>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
with tessract engine trained
</commit_message>
<xml_diff>
--- a/invoice_data.xlsx
+++ b/invoice_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,53 +413,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>filename</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Invoice No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Invoice Date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Dealer Code</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Sale Order</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Vender Code</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Vehicle Code</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>02.jpg</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>05-rotat.jpg</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>05.jpg</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>28.02.2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PPR8</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10.jpg</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0000000000</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>